<commit_message>
update on mithi demand
</commit_message>
<xml_diff>
--- a/client-side/uploads/template.xlsx
+++ b/client-side/uploads/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nullbyte00_/Developer/archived_proj/pieds/MassMailingCC/client-side/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680323FD-6C16-F148-A444-A85EAF32C6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8F82514-645A-B245-9CDC-448AD8670806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="21340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="36000" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>Designation</t>
   </si>
@@ -37,52 +37,55 @@
     <t>Email</t>
   </si>
   <si>
-    <t>A_Designation</t>
-  </si>
-  <si>
-    <t>B_Designation</t>
-  </si>
-  <si>
     <t>Event Organizer</t>
   </si>
   <si>
-    <t>EVENT1</t>
+    <t>Srijan</t>
   </si>
   <si>
-    <t>EVENT2</t>
+    <t>Sahay</t>
   </si>
   <si>
-    <t>Shanker</t>
+    <t>PIEDS Student Team</t>
   </si>
   <si>
-    <t>Saini</t>
+    <t>f20240829@pilani.bits-pilani.ac.in</t>
   </si>
   <si>
-    <t>Harshit</t>
+    <t>f20240474@pilani.bits-pilani.ac.in</t>
   </si>
   <si>
-    <t>CVR</t>
+    <t>Harhsit</t>
   </si>
   <si>
-    <t>Himanshu</t>
+    <t>Jiya</t>
   </si>
   <si>
-    <t>f20221355@pilani.bits-pilani.ac.in</t>
+    <t>f20240868@pilani.bits-pilani.ac.in</t>
   </si>
   <si>
-    <t>RKIC</t>
+    <t>Krrish</t>
   </si>
   <si>
-    <t xml:space="preserve">Swasti </t>
+    <t>f20241019@pilani.bits-pilani.ac.in</t>
   </si>
   <si>
-    <t>Dubey</t>
+    <t>Sarvesh</t>
   </si>
   <si>
-    <t>f20231237@pilani.bits-pilani.ac.in</t>
+    <t>f20240996@pilani.bits-pilani.ac.in</t>
   </si>
   <si>
-    <t>f20240474@pilani.bits-pilani.ac.in,f20240996@pilani.bits-pilani.ac.in</t>
+    <t>Shreyashi</t>
+  </si>
+  <si>
+    <t>f20240339@pilani.bits-pilani.ac.in</t>
+  </si>
+  <si>
+    <t>Tushar</t>
+  </si>
+  <si>
+    <t>f20241053@pilani.bits-pilani.ac.in</t>
   </si>
 </sst>
 </file>
@@ -414,7 +417,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="1"/>
@@ -439,23 +442,19 @@
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
+      <c r="D2" s="2"/>
+      <c r="E2" s="4" t="s">
+        <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="F2" s="2"/>
       <c r="G2" s="4"/>
       <c r="H2" s="2"/>
       <c r="I2" s="3"/>
@@ -478,23 +477,17 @@
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="4" t="s">
+        <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="F3" s="2"/>
       <c r="G3" s="4"/>
       <c r="H3" s="2"/>
       <c r="I3" s="3"/>
@@ -517,17 +510,15 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="4" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="4"/>
@@ -551,11 +542,17 @@
       <c r="Y4" s="2"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F5" s="2"/>
       <c r="G5" s="4"/>
       <c r="H5" s="2"/>
@@ -578,11 +575,17 @@
       <c r="Y5" s="2"/>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="4"/>
       <c r="H6" s="2"/>
@@ -605,11 +608,17 @@
       <c r="Y6" s="2"/>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="4"/>
       <c r="H7" s="2"/>
@@ -632,11 +641,17 @@
       <c r="Y7" s="2"/>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="4"/>
+      <c r="E8" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="4"/>
       <c r="H8" s="2"/>
@@ -3435,9 +3450,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{882F5B68-2F2E-A545-91B4-F5B89B48D154}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{36CD0EA5-0D29-BC4F-ABDB-2F710839319C}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{42D4C088-4CD1-A640-AE71-17CE24BCDBE0}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{8AE62794-AAC4-3E4E-A6D2-94BE0C1C9F42}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>